<commit_message>
fix: support ACCESO column header variant from Excel template
The template uses "ACCESO (USO/CONSULTA)" as header but code only
checked "ACCESO". Now accepts both variants. Also updated Referencias
sheet with ACCESO documentation.

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/Tolvink_-_Modelo_carga.xlsx
+++ b/public/Tolvink_-_Modelo_carga.xlsx
@@ -399,15 +399,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <cols>
-    <col min="1" max="1" width="25.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
-    <col min="3" max="3" width="25.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="18.83203125" customWidth="1"/>
-    <col min="6" max="6" width="14.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -417,15 +409,18 @@
         <v>TIPO</v>
       </c>
       <c r="C1" t="str">
+        <v>ACCESO (USO/CONSULTA)</v>
+      </c>
+      <c r="D1" t="str">
         <v>EMAIL</v>
       </c>
-      <c r="D1" t="str">
+      <c r="E1" t="str">
         <v>TELEFONO</v>
       </c>
-      <c r="E1" t="str">
+      <c r="F1" t="str">
         <v>RUT</v>
       </c>
-      <c r="F1" t="str">
+      <c r="G1" t="str">
         <v>FLOTA PROPIA</v>
       </c>
     </row>
@@ -437,15 +432,18 @@
         <v>PLANTA</v>
       </c>
       <c r="C2" t="str">
+        <v>USO</v>
+      </c>
+      <c r="D2" t="str">
         <v>planta@ejemplo.com</v>
       </c>
-      <c r="D2" t="str">
+      <c r="E2" t="str">
         <v>099123456</v>
       </c>
-      <c r="E2" t="str">
+      <c r="F2" t="str">
         <v>210000000012</v>
       </c>
-      <c r="F2" t="str">
+      <c r="G2" t="str">
         <v>NO</v>
       </c>
     </row>
@@ -457,36 +455,32 @@
         <v>PRODUCTOR</v>
       </c>
       <c r="C3" t="str">
+        <v>CONSULTA</v>
+      </c>
+      <c r="D3" t="str">
         <v>prod@ejemplo.com</v>
       </c>
-      <c r="D3" t="str">
+      <c r="E3" t="str">
         <v>099654321</v>
       </c>
-      <c r="E3" t="str">
+      <c r="F3" t="str">
         <v>210000000013</v>
       </c>
-      <c r="F3" t="str">
+      <c r="G3" t="str">
         <v>SI</v>
       </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F3"/>
-  <cols>
-    <col min="1" max="1" width="22.83203125" customWidth="1"/>
-    <col min="2" max="2" width="25.83203125" customWidth="1"/>
-    <col min="3" max="3" width="15.83203125" customWidth="1"/>
-    <col min="4" max="4" width="15.83203125" customWidth="1"/>
-    <col min="5" max="5" width="25.83203125" customWidth="1"/>
-    <col min="6" max="6" width="12.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:G3"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -507,6 +501,9 @@
       <c r="F1" t="str">
         <v>ROL</v>
       </c>
+      <c r="G1" t="str">
+        <v>ACCESO (USO/CONSULTA)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -527,6 +524,9 @@
       <c r="F2" t="str">
         <v>GERENTE</v>
       </c>
+      <c r="G2" t="str">
+        <v>USO</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -547,21 +547,21 @@
       <c r="F3" t="str">
         <v>OPERARIO</v>
       </c>
+      <c r="G3" t="str">
+        <v>CONSULTA</v>
+      </c>
     </row>
   </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:F3"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G3"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
-  <cols>
-    <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="55.83203125" customWidth="1"/>
-  </cols>
+  <dimension ref="A1:B7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
@@ -581,39 +581,47 @@
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>FLOTA PROPIA</v>
+        <v>ACCESO</v>
       </c>
       <c r="B3" t="str">
-        <v>SI, NO (default: NO)</v>
+        <v>USO, CONSULTA (obligatorio)</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>ROL (usuario)</v>
+        <v>FLOTA PROPIA</v>
       </c>
       <c r="B4" t="str">
-        <v>OPERARIO, GERENTE, CHOFER</v>
+        <v>SI, NO (default: NO)</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>CONTRASEÑA</v>
+        <v>ROL (usuario)</v>
       </c>
       <c r="B5" t="str">
-        <v>Mínimo 8 caracteres, 1 mayúscula, 1 minúscula, 1 número</v>
+        <v>OPERARIO, GERENTE, CHOFER</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
+        <v>CONTRASEÑA</v>
+      </c>
+      <c r="B6" t="str">
+        <v>Mínimo 6 caracteres</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
         <v>EMPRESA (usuario)</v>
       </c>
-      <c r="B6" t="str">
+      <c r="B7" t="str">
         <v>Debe coincidir EXACTO con el nombre de una empresa existente</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>